<commit_message>
add subject mandatory bp (#76) de85eaccf4ace281cecaadda1ed0266ae8e6f06f
</commit_message>
<xml_diff>
--- a/ig/main/StructureDefinition-mesures-fr-observation-bmi.xlsx
+++ b/ig/main/StructureDefinition-mesures-fr-observation-bmi.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2023-11-23T10:14:09+00:00</t>
+    <t>2023-11-28T12:14:54+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -440,11 +440,10 @@
 </t>
   </si>
   <si>
-    <t>Uri identifiant les systèmes tiers ayant envoyé la ressource.</t>
-  </si>
-  <si>
-    <t>Uri identifiant les systèmes tiers ayant envoyé la ressource.
-L’uri est sous la forme d’un oid : « urn:oid:xx.xx.xx »</t>
+    <t>Uri identifiant les systèmes tiers ayant envoyé la ressource. L’uri est sous la forme d’une oid : « urn:oid:xx.xx.xx »</t>
+  </si>
+  <si>
+    <t>A uri that identifies the source system of the resource. This provides a minimal amount of [Provenance](provenance.html#) information that can be used to track or differentiate the source of information in the resource. The source may identify another FHIR server, document, message, database, etc.</t>
   </si>
   <si>
     <t>In the provenance resource, this corresponds to Provenance.entity.what[x]. The exact use of the source (and the implied Provenance.entity.role) is left to implementer discretion. Only one nominated source is allowed; for additional provenance details, a full Provenance resource should be used. 

</xml_diff>

<commit_message>
update MDC terminology descr d1f6467a37bcf0dec3dae5b61eebe8ba055be48d
</commit_message>
<xml_diff>
--- a/ig/main/StructureDefinition-mesures-fr-observation-bmi.xlsx
+++ b/ig/main/StructureDefinition-mesures-fr-observation-bmi.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2023-11-28T13:07:26+00:00</t>
+    <t>2023-11-28T13:18:47+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -12326,7 +12326,7 @@
         <v>91</v>
       </c>
       <c r="H82" t="s" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="I82" t="s" s="2">
         <v>80</v>

</xml_diff>